<commit_message>
Fixing the mistakes Efficient SU2 and Adding new custom quantum kernel
</commit_message>
<xml_diff>
--- a/results/combined_results.xlsx
+++ b/results/combined_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\qq\QML\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30892E95-F822-4D58-827F-EDA5B33FB325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF568C44-9921-4EDD-B419-0A1BAF76F1B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2625" yWindow="2715" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5205" yWindow="4365" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Accuracy</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>Efficient_SU2</t>
+  </si>
+  <si>
+    <t>Custom hybrid Angle-Phase quantum feature map with entanglement layers</t>
   </si>
 </sst>
 </file>
@@ -384,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -549,31 +552,63 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>0.90518553000000002</v>
+        <v>0.97188324800000003</v>
       </c>
       <c r="C6">
-        <v>0.93334718400000005</v>
+        <v>0.97139108900000004</v>
       </c>
       <c r="D6">
-        <v>0.80199335500000002</v>
+        <v>0.95282392000000005</v>
       </c>
       <c r="E6">
-        <v>0.86133194099999999</v>
+        <v>0.96183272099999995</v>
       </c>
       <c r="F6">
-        <v>0.89295293799999997</v>
+        <v>0.972482238</v>
       </c>
       <c r="G6">
-        <v>0.96635367800000005</v>
+        <v>0.98317683899999997</v>
       </c>
       <c r="H6">
-        <v>0.92787481000000005</v>
+        <v>0.97773609100000003</v>
       </c>
       <c r="I6">
-        <v>0.89460337499999998</v>
+        <v>0.96978440600000004</v>
       </c>
       <c r="J6">
-        <v>0.88417351700000002</v>
+        <v>0.96800037999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>0.97365315900000005</v>
+      </c>
+      <c r="C7">
+        <v>0.97248629200000003</v>
+      </c>
+      <c r="D7">
+        <v>0.95747508299999995</v>
+      </c>
+      <c r="E7">
+        <v>0.964621752</v>
+      </c>
+      <c r="F7">
+        <v>0.97510333699999996</v>
+      </c>
+      <c r="G7">
+        <v>0.98313771500000002</v>
+      </c>
+      <c r="H7">
+        <v>0.97899647700000003</v>
+      </c>
+      <c r="I7">
+        <v>0.97180911400000003</v>
+      </c>
+      <c r="J7">
+        <v>0.97030639900000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding Data scaling in preprocess of classical kernels
</commit_message>
<xml_diff>
--- a/results/combined_results.xlsx
+++ b/results/combined_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\qq\QML\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF568C44-9921-4EDD-B419-0A1BAF76F1B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FA4B85-81E5-4309-AF43-5F4FB8F72288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5205" yWindow="4365" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -424,31 +424,31 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>0.95255395099999995</v>
+        <v>0.97362210836826502</v>
       </c>
       <c r="C2">
-        <v>0.94715447200000003</v>
+        <v>0.99</v>
       </c>
       <c r="D2">
-        <v>0.92436323399999998</v>
+        <v>0.93864894795127296</v>
       </c>
       <c r="E2">
-        <v>0.93530689099999997</v>
+        <v>0.963557312303574</v>
       </c>
       <c r="F2">
-        <v>0.95618758999999998</v>
+        <v>0.96478682792381398</v>
       </c>
       <c r="G2">
-        <v>0.96917057900000003</v>
+        <v>0.99436619718309804</v>
       </c>
       <c r="H2">
-        <v>0.96252101800000001</v>
+        <v>0.97932793264124596</v>
       </c>
       <c r="I2">
-        <v>0.948913954</v>
+        <v>0.97144262247240998</v>
       </c>
       <c r="J2">
-        <v>0.94676690600000002</v>
+        <v>0.966507572567186</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -456,31 +456,31 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>0.92100605499999999</v>
+        <v>0.98065517776742706</v>
       </c>
       <c r="C3">
-        <v>0.96819887400000004</v>
+        <v>0.99024390243902405</v>
       </c>
       <c r="D3">
-        <v>0.816057586</v>
+        <v>0.95758582502768497</v>
       </c>
       <c r="E3">
-        <v>0.88301416300000002</v>
+        <v>0.97355067328136002</v>
       </c>
       <c r="F3">
-        <v>0.90200976799999999</v>
+        <v>0.97533938047636604</v>
       </c>
       <c r="G3">
-        <v>0.98309859200000005</v>
+        <v>0.99440532081377098</v>
       </c>
       <c r="H3">
-        <v>0.94024630600000003</v>
+        <v>0.98475042199180096</v>
       </c>
       <c r="I3">
-        <v>0.91163023499999996</v>
+        <v>0.97915054763658105</v>
       </c>
       <c r="J3">
-        <v>0.89957808900000003</v>
+        <v>0.97599557292072803</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -488,31 +488,31 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>0.91221859999999999</v>
+        <v>0.97540754541220298</v>
       </c>
       <c r="C4">
-        <v>0.96135540500000005</v>
+        <v>0.98571428571428499</v>
       </c>
       <c r="D4">
-        <v>0.79712070899999998</v>
+        <v>0.94828349944628998</v>
       </c>
       <c r="E4">
-        <v>0.86935686300000004</v>
+        <v>0.96648837613211602</v>
       </c>
       <c r="F4">
-        <v>0.89229705699999995</v>
+        <v>0.96993084633929705</v>
       </c>
       <c r="G4">
-        <v>0.98032081400000004</v>
+        <v>0.99154929577464701</v>
       </c>
       <c r="H4">
-        <v>0.93378214000000004</v>
+        <v>0.98057270850926503</v>
       </c>
       <c r="I4">
-        <v>0.90156950199999997</v>
+        <v>0.97353054232069003</v>
       </c>
       <c r="J4">
-        <v>0.88872076099999997</v>
+        <v>0.96991639761046899</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -520,31 +520,31 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>0.44977487999999999</v>
+        <v>0.30929979816798597</v>
       </c>
       <c r="C5">
-        <v>0.206400899</v>
+        <v>1.98290598290598E-2</v>
       </c>
       <c r="D5">
-        <v>0.165227021</v>
+        <v>1.8715393133997699E-2</v>
       </c>
       <c r="E5">
-        <v>0.18045538799999999</v>
+        <v>1.9231847490888701E-2</v>
       </c>
       <c r="F5">
-        <v>0.55318793099999997</v>
+        <v>0.45126107091147999</v>
       </c>
       <c r="G5">
-        <v>0.61948356800000004</v>
+        <v>0.48204225352112601</v>
       </c>
       <c r="H5">
-        <v>0.58276877100000002</v>
+        <v>0.46569587731482798</v>
       </c>
       <c r="I5">
-        <v>0.38161207899999999</v>
+        <v>0.242463862402858</v>
       </c>
       <c r="J5">
-        <v>0.39235529499999999</v>
+        <v>0.25037882332756201</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>